<commit_message>
Try and preempt row height based on content being translated
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/csoc/02-csoc-prn-obligations-home.xlsx
+++ b/translations/welsh-translations/csoc/02-csoc-prn-obligations-home.xlsx
@@ -735,7 +735,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
+    <row r="20" ht="51" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_ObligationsHome.en.resx::cancelled_paragraph_compliance_scheme</t>
@@ -777,7 +777,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
+    <row r="21" ht="51" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_ObligationsHome.en.resx::cancelled_paragraph_direct_producer</t>

</xml_diff>